<commit_message>
Fix device summary report column format
</commit_message>
<xml_diff>
--- a/api/templates/device_summary_report/en.xlsx
+++ b/api/templates/device_summary_report/en.xlsx
@@ -95,11 +95,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm"/>
-    <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -218,7 +217,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -227,15 +226,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -259,6 +258,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -267,11 +270,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -352,32 +359,25 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:AMJ12"/>
   <sheetFormatPr defaultColWidth="11.21484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="40.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="31.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="6" style="1" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="14.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="3" width="14.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="12" style="2" width="14.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="13.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="10.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="2" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="3" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1015" style="1" width="9.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="27.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1008" min="999" style="1" width="9.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16369" style="0" width="9.34"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -423,11 +423,11 @@
       <c r="C8" s="8"/>
       <c r="D8" s="7"/>
     </row>
-    <row r="9" s="10" customFormat="true" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" s="11" customFormat="true" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -436,58 +436,42 @@
       <c r="D9" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="0"/>
-      <c r="F9" s="0"/>
-      <c r="G9" s="0"/>
-      <c r="H9" s="0"/>
-      <c r="I9" s="0"/>
-      <c r="J9" s="0"/>
-      <c r="K9" s="0"/>
-      <c r="L9" s="0"/>
-      <c r="M9" s="0"/>
-      <c r="N9" s="0"/>
-      <c r="O9" s="0"/>
-      <c r="P9" s="0"/>
-      <c r="Q9" s="0"/>
-      <c r="R9" s="0"/>
-      <c r="S9" s="0"/>
-      <c r="T9" s="0"/>
+      <c r="ALU9" s="0"/>
+      <c r="ALV9" s="0"/>
+      <c r="ALW9" s="0"/>
+      <c r="ALX9" s="0"/>
+      <c r="ALY9" s="0"/>
+      <c r="ALZ9" s="0"/>
+      <c r="AMA9" s="0"/>
+      <c r="AMB9" s="0"/>
+      <c r="AMC9" s="0"/>
+      <c r="AMD9" s="0"/>
+      <c r="AME9" s="0"/>
+      <c r="AMF9" s="0"/>
+      <c r="AMG9" s="0"/>
+      <c r="AMH9" s="0"/>
+      <c r="AMI9" s="0"/>
+      <c r="AMJ9" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="0"/>
-      <c r="F10" s="0"/>
-      <c r="G10" s="0"/>
-      <c r="H10" s="0"/>
-      <c r="I10" s="0"/>
-      <c r="J10" s="0"/>
-      <c r="K10" s="0"/>
-      <c r="L10" s="0"/>
-      <c r="M10" s="0"/>
-      <c r="N10" s="0"/>
-      <c r="O10" s="0"/>
-      <c r="P10" s="0"/>
-      <c r="Q10" s="0"/>
-      <c r="R10" s="0"/>
-      <c r="S10" s="0"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>